<commit_message>
modified passing and average thresholds for A1, A2 and B1
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Neil\Desktop\generate_reports_project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BAF1512-C0D8-4991-8A8A-8CF182DA24AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0630B72-A68A-4965-9818-2F9731D5EB83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20544" yWindow="0" windowWidth="20832" windowHeight="16656" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1248" yWindow="1248" windowWidth="30960" windowHeight="12168" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Students" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
   <si>
     <t>B2</t>
   </si>
@@ -70,13 +70,22 @@
   </si>
   <si>
     <t>CERTIFICATION</t>
+  </si>
+  <si>
+    <t>dfsdaf</t>
+  </si>
+  <si>
+    <t>fgsdfgsdfg</t>
+  </si>
+  <si>
+    <t>dgfadsfgsdfg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -88,6 +97,12 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -131,6 +146,22 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7485F647-8EE1-4C4F-B49E-95899FF2CD53}" name="Table1" displayName="Table1" ref="A1:G8" totalsRowShown="0">
+  <autoFilter ref="A1:G8" xr:uid="{7485F647-8EE1-4C4F-B49E-95899FF2CD53}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{C5E00F0E-939E-49D3-80A9-FC11FDBBAD1E}" name="STUDENT"/>
+    <tableColumn id="2" xr3:uid="{D0D5AFD9-A45E-4EB1-8F59-9BD146B2EC32}" name="EXAMS DONE"/>
+    <tableColumn id="3" xr3:uid="{A3F26F88-842C-4302-A3D8-A6A247DFA697}" name="CERTIFICATION"/>
+    <tableColumn id="4" xr3:uid="{56E3D525-B45A-4EB1-9727-4A62D4EBFE93}" name="READING"/>
+    <tableColumn id="5" xr3:uid="{EB77B100-CCBB-42A6-84CC-144320CF5143}" name="USE OF ENGLISH"/>
+    <tableColumn id="6" xr3:uid="{E6031C17-D40D-4ACF-BFFF-9B09674DC54C}" name="WRITING"/>
+    <tableColumn id="7" xr3:uid="{68117322-CF51-44AC-9D09-082E8C34F369}" name="LISTENING"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -397,13 +428,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
     <col min="2" max="2" width="23.42578125" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" customWidth="1"/>
-    <col min="5" max="5" width="17" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="17.140625" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -521,17 +554,90 @@
         <v>34</v>
       </c>
     </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>65</v>
+      </c>
+      <c r="E6">
+        <v>65</v>
+      </c>
+      <c r="F6">
+        <v>65</v>
+      </c>
+      <c r="G6">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7">
+        <v>55</v>
+      </c>
+      <c r="E7">
+        <v>55</v>
+      </c>
+      <c r="F7">
+        <v>55</v>
+      </c>
+      <c r="G7">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8">
+        <v>75</v>
+      </c>
+      <c r="E8">
+        <v>75</v>
+      </c>
+      <c r="F8">
+        <v>75</v>
+      </c>
+      <c r="G8">
+        <v>75</v>
+      </c>
+    </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
       <c r="E9" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C5" xr:uid="{132590E1-DD2B-4538-A8F6-64A79E2FFEBD}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C8" xr:uid="{132590E1-DD2B-4538-A8F6-64A79E2FFEBD}">
       <formula1>"A1, A2, B1, B2, C1, C2"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>